<commit_message>
feat: fake data preparation
</commit_message>
<xml_diff>
--- a/Data Dictionary CollectAI.xlsx
+++ b/Data Dictionary CollectAI.xlsx
@@ -4,15 +4,15 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000" firstSheet="2" activeTab="2"/>
+    <workbookView windowHeight="14740" firstSheet="2" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Customer Master" sheetId="1" r:id="rId1"/>
     <sheet name="Contract Snapshot" sheetId="2" r:id="rId2"/>
     <sheet name="Payment History" sheetId="3" r:id="rId3"/>
     <sheet name="LKP &amp; Interaction History" sheetId="4" r:id="rId4"/>
-    <sheet name="AI Intelligence Output" sheetId="5" r:id="rId5"/>
-    <sheet name="Customer Behavioral Standing" sheetId="6" r:id="rId6"/>
+    <sheet name="Collection Analysis" sheetId="5" r:id="rId5"/>
+    <sheet name="Customer Analysis" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="111">
   <si>
     <t>Field Name</t>
   </si>
@@ -262,6 +262,9 @@
     <t>Optional, Range: 1-5</t>
   </si>
   <si>
+    <t>FK Customer Master</t>
+  </si>
+  <si>
     <t>RECOVERY_SCORE</t>
   </si>
   <si>
@@ -298,10 +301,22 @@
     <t>Optional, Decimal</t>
   </si>
   <si>
-    <t>LAST_CONTRACT_NO</t>
+    <t>SCORING_DATE</t>
+  </si>
+  <si>
+    <t>Tanggal Scoring Dilakukan</t>
+  </si>
+  <si>
+    <t>ACTIVE_CONTRACT_COUNT</t>
   </si>
   <si>
     <t>Nomor kontrak terakhir yang diselesaikan.</t>
+  </si>
+  <si>
+    <t>TOTAL_ACTIVE_OTS</t>
+  </si>
+  <si>
+    <t>SUM(PRNC_OTS + INTR_OTS) semua kontrak aktif</t>
   </si>
   <si>
     <t>BEHAVIORAL_GRADE</t>
@@ -362,14 +377,7 @@
     <numFmt numFmtId="178" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="179" formatCode="_-&quot;Rp&quot;* #,##0_-;\-&quot;Rp&quot;* #,##0_-;_-&quot;Rp&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="21">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -825,148 +833,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -980,12 +988,12 @@
     <cellStyle name="Percent" xfId="3" builtinId="5"/>
     <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
     <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
     <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
     <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
     <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
     <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
     <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
@@ -1319,12 +1327,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="7" outlineLevelCol="3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="7" outlineLevelCol="3"/>
   <cols>
-    <col min="1" max="1" width="21.1111111111111" customWidth="1"/>
-    <col min="2" max="2" width="9.88888888888889" customWidth="1"/>
-    <col min="3" max="3" width="47.1111111111111" customWidth="1"/>
-    <col min="4" max="4" width="21.5555555555556" customWidth="1"/>
+    <col min="1" max="1" width="21.109375" customWidth="1"/>
+    <col min="2" max="2" width="9.890625" customWidth="1"/>
+    <col min="3" max="3" width="47.109375" customWidth="1"/>
+    <col min="4" max="4" width="21.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -1449,12 +1457,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="7" outlineLevelCol="3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="7" outlineLevelCol="3"/>
   <cols>
-    <col min="1" max="1" width="15.4444444444444" customWidth="1"/>
-    <col min="2" max="2" width="9.88888888888889" customWidth="1"/>
-    <col min="3" max="3" width="101.666666666667" customWidth="1"/>
-    <col min="4" max="4" width="21.5555555555556" customWidth="1"/>
+    <col min="1" max="1" width="15.4453125" customWidth="1"/>
+    <col min="2" max="2" width="9.890625" customWidth="1"/>
+    <col min="3" max="3" width="101.6640625" customWidth="1"/>
+    <col min="4" max="4" width="21.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -1579,11 +1587,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:D9"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="3"/>
   <cols>
-    <col min="1" max="1" width="19.6666666666667" customWidth="1"/>
-    <col min="2" max="2" width="9.88888888888889" customWidth="1"/>
-    <col min="3" max="3" width="50.2222222222222" customWidth="1"/>
+    <col min="1" max="1" width="19.6640625" customWidth="1"/>
+    <col min="2" max="2" width="9.890625" customWidth="1"/>
+    <col min="3" max="3" width="50.21875" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1723,11 +1731,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:D9"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="3"/>
   <cols>
-    <col min="1" max="1" width="20.7777777777778" customWidth="1"/>
-    <col min="2" max="2" width="9.88888888888889" customWidth="1"/>
-    <col min="3" max="3" width="59.2222222222222" customWidth="1"/>
+    <col min="1" max="1" width="20.78125" customWidth="1"/>
+    <col min="2" max="2" width="9.890625" customWidth="1"/>
+    <col min="3" max="3" width="59.21875" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1866,12 +1874,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="6" outlineLevelCol="3"/>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="3"/>
   <cols>
-    <col min="1" max="1" width="24.6666666666667" customWidth="1"/>
-    <col min="2" max="2" width="9.88888888888889" customWidth="1"/>
-    <col min="3" max="3" width="52.8888888888889" customWidth="1"/>
+    <col min="1" max="1" width="24.6640625" customWidth="1"/>
+    <col min="2" max="2" width="9.890625" customWidth="1"/>
+    <col min="3" max="3" width="52.890625" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1905,41 +1913,41 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
         <v>76</v>
       </c>
-      <c r="B3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" t="s">
-        <v>77</v>
-      </c>
       <c r="D3" t="s">
-        <v>78</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C4" t="s">
+        <v>78</v>
+      </c>
+      <c r="D4" t="s">
         <v>79</v>
-      </c>
-      <c r="B4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" t="s">
-        <v>80</v>
-      </c>
-      <c r="D4" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
+        <v>80</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
         <v>81</v>
-      </c>
-      <c r="B5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" t="s">
-        <v>82</v>
       </c>
       <c r="D5" t="s">
         <v>38</v>
@@ -1947,13 +1955,13 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
+        <v>82</v>
+      </c>
+      <c r="B6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
         <v>83</v>
-      </c>
-      <c r="B6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" t="s">
-        <v>84</v>
       </c>
       <c r="D6" t="s">
         <v>38</v>
@@ -1961,16 +1969,44 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
+        <v>84</v>
+      </c>
+      <c r="B7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
         <v>85</v>
       </c>
-      <c r="B7" t="s">
+      <c r="D7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" t="s">
+        <v>86</v>
+      </c>
+      <c r="B8" t="s">
         <v>32</v>
       </c>
-      <c r="C7" t="s">
-        <v>86</v>
-      </c>
-      <c r="D7" t="s">
+      <c r="C8" t="s">
         <v>87</v>
+      </c>
+      <c r="D8" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" t="s">
+        <v>89</v>
+      </c>
+      <c r="B9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" t="s">
+        <v>90</v>
+      </c>
+      <c r="D9" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -1982,13 +2018,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D9"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="3"/>
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="3"/>
   <cols>
-    <col min="1" max="1" width="25.2222222222222" customWidth="1"/>
-    <col min="2" max="2" width="10.7777777777778" customWidth="1"/>
-    <col min="3" max="3" width="54.2222222222222" customWidth="1"/>
-    <col min="4" max="4" width="24.6666666666667" customWidth="1"/>
+    <col min="1" max="1" width="25.21875" customWidth="1"/>
+    <col min="2" max="2" width="10.78125" customWidth="1"/>
+    <col min="3" max="3" width="54.21875" customWidth="1"/>
+    <col min="4" max="4" width="24.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -2021,13 +2057,13 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D3" t="s">
         <v>27</v>
@@ -2035,27 +2071,27 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C4" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D4" t="s">
-        <v>38</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B5" t="s">
         <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D5" t="s">
         <v>38</v>
@@ -2063,58 +2099,72 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B6" t="s">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="D6" t="s">
-        <v>78</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B7" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C7" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D7" t="s">
-        <v>14</v>
+        <v>79</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B8" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
       <c r="C8" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D8" t="s">
-        <v>101</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D9" t="s">
-        <v>105</v>
+        <v>106</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" t="s">
+        <v>107</v>
+      </c>
+      <c r="B10" t="s">
+        <v>108</v>
+      </c>
+      <c r="C10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D10" t="s">
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: self improving pipeline
</commit_message>
<xml_diff>
--- a/Data Dictionary CollectAI.xlsx
+++ b/Data Dictionary CollectAI.xlsx
@@ -4,15 +4,15 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="14740" firstSheet="2" activeTab="5"/>
+    <workbookView windowHeight="16360" firstSheet="2" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Customer Master" sheetId="1" r:id="rId1"/>
     <sheet name="Contract Snapshot" sheetId="2" r:id="rId2"/>
     <sheet name="Payment History" sheetId="3" r:id="rId3"/>
     <sheet name="LKP &amp; Interaction History" sheetId="4" r:id="rId4"/>
-    <sheet name="Collection Analysis" sheetId="5" r:id="rId5"/>
-    <sheet name="Customer Analysis" sheetId="6" r:id="rId6"/>
+    <sheet name="AI Intelligence Output" sheetId="5" r:id="rId5"/>
+    <sheet name="Customer Behavioral Standing" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="113">
   <si>
     <t>Field Name</t>
   </si>
@@ -274,6 +274,21 @@
     <t>Mandatory, Decimal</t>
   </si>
   <si>
+    <t>CONFIDENCE_CATEGORY</t>
+  </si>
+  <si>
+    <t>Kategori tingkat keyakinan AI terhadap rekomendasi NBA.</t>
+  </si>
+  <si>
+    <t>CONFIDENCE_LEVEL</t>
+  </si>
+  <si>
+    <t>Tingkat keyakinan AI terhadap rekomendasi NBA.</t>
+  </si>
+  <si>
+    <t>Optional, Decimal</t>
+  </si>
+  <si>
     <t>RISK_SEGMENT</t>
   </si>
   <si>
@@ -290,15 +305,6 @@
   </si>
   <si>
     <t>Urutan kerja collector: Critical, High, Medium, Low.</t>
-  </si>
-  <si>
-    <t>CONFIDENCE_LEVEL</t>
-  </si>
-  <si>
-    <t>Tingkat keyakinan AI terhadap rekomendasi NBA.</t>
-  </si>
-  <si>
-    <t>Optional, Decimal</t>
   </si>
   <si>
     <t>SCORING_DATE</t>
@@ -1874,7 +1880,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="24.6640625" customWidth="1"/>
@@ -1950,7 +1956,7 @@
         <v>81</v>
       </c>
       <c r="D5" t="s">
-        <v>38</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -1958,24 +1964,24 @@
         <v>82</v>
       </c>
       <c r="B6" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C6" t="s">
         <v>83</v>
       </c>
       <c r="D6" t="s">
-        <v>38</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B7" t="s">
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D7" t="s">
         <v>38</v>
@@ -1983,16 +1989,16 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B8" t="s">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="C8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D8" t="s">
-        <v>88</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -2000,12 +2006,26 @@
         <v>89</v>
       </c>
       <c r="B9" t="s">
-        <v>46</v>
+        <v>5</v>
       </c>
       <c r="C9" t="s">
         <v>90</v>
       </c>
       <c r="D9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" t="s">
+        <v>91</v>
+      </c>
+      <c r="B10" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10" t="s">
+        <v>92</v>
+      </c>
+      <c r="D10" t="s">
         <v>48</v>
       </c>
     </row>
@@ -2057,13 +2077,13 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D3" t="s">
         <v>27</v>
@@ -2071,13 +2091,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B4" t="s">
         <v>32</v>
       </c>
       <c r="C4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D4" t="s">
         <v>79</v>
@@ -2085,13 +2105,13 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B5" t="s">
         <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D5" t="s">
         <v>38</v>
@@ -2099,13 +2119,13 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B6" t="s">
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D6" t="s">
         <v>38</v>
@@ -2113,13 +2133,13 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B7" t="s">
         <v>32</v>
       </c>
       <c r="C7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D7" t="s">
         <v>79</v>
@@ -2127,13 +2147,13 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B8" t="s">
         <v>5</v>
       </c>
       <c r="C8" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D8" t="s">
         <v>14</v>
@@ -2141,30 +2161,30 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B9" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C9" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D9" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B10" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C10" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D10" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>